<commit_message>
fix bug excel file
</commit_message>
<xml_diff>
--- a/static/docs/sample_import.xlsx
+++ b/static/docs/sample_import.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wilmer.acosta/sources/retail-foundry/static/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AABF647F-14BC-2B47-9624-2D64A884857E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D384D71D-5A03-E046-9F36-2D33E2A8E9F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34380" yWindow="7180" windowWidth="36480" windowHeight="17200" xr2:uid="{813F6D71-8612-0742-B7C7-BC465FB9967B}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="17200" activeTab="2" xr2:uid="{813F6D71-8612-0742-B7C7-BC465FB9967B}"/>
   </bookViews>
   <sheets>
     <sheet name="Localidades" sheetId="1" r:id="rId1"/>
-    <sheet name="Competencias" sheetId="2" r:id="rId2"/>
+    <sheet name="Competidores" sheetId="2" r:id="rId2"/>
     <sheet name="Canibalizadores" sheetId="3" r:id="rId3"/>
     <sheet name="Tipos de Datos" sheetId="4" r:id="rId4"/>
   </sheets>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
   <si>
     <t>ID</t>
   </si>
@@ -47,12 +47,6 @@
     <t>Nombre</t>
   </si>
   <si>
-    <t>Tipo de Localidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tamaño (m²) </t>
-  </si>
-  <si>
     <t>Latitud</t>
   </si>
   <si>
@@ -62,12 +56,6 @@
     <t>Zona de Movilidad</t>
   </si>
   <si>
-    <t>Hogares a 5min</t>
-  </si>
-  <si>
-    <t>Hogares a 10min</t>
-  </si>
-  <si>
     <t>% NSE D</t>
   </si>
   <si>
@@ -113,12 +101,6 @@
     <t>Zona alta</t>
   </si>
   <si>
-    <t>ID de Localidad</t>
-  </si>
-  <si>
-    <t>Tipo de Competidor</t>
-  </si>
-  <si>
     <t>Provincia</t>
   </si>
   <si>
@@ -129,6 +111,21 @@
   </si>
   <si>
     <t>Dirección</t>
+  </si>
+  <si>
+    <t>Tipo</t>
+  </si>
+  <si>
+    <t>Hogares 10min</t>
+  </si>
+  <si>
+    <t>Hogares 5min</t>
+  </si>
+  <si>
+    <t>Localidad ID</t>
+  </si>
+  <si>
+    <t>Tamaño</t>
   </si>
 </sst>
 </file>
@@ -272,8 +269,8 @@
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{B22F800C-EB91-0945-8005-2E58916CFD1A}" name="ID"/>
     <tableColumn id="2" xr3:uid="{1AFD6444-6C83-E442-BC36-F2D8A848BC0F}" name="Nombre"/>
-    <tableColumn id="3" xr3:uid="{07AB825C-731B-1C43-BC3C-E14E7C9172A7}" name="Tipo de Localidad"/>
-    <tableColumn id="4" xr3:uid="{22E95836-6AA5-3745-9BA6-02A87D3166B1}" name="Tamaño (m²) "/>
+    <tableColumn id="3" xr3:uid="{07AB825C-731B-1C43-BC3C-E14E7C9172A7}" name="Tipo"/>
+    <tableColumn id="4" xr3:uid="{22E95836-6AA5-3745-9BA6-02A87D3166B1}" name="Tamaño"/>
     <tableColumn id="5" xr3:uid="{E33C6D42-A2E8-544F-B029-5BB889BE05AE}" name="Latitud"/>
     <tableColumn id="6" xr3:uid="{B6260D0E-41D6-CB4F-A132-020FC93AD441}" name="Longitud"/>
     <tableColumn id="17" xr3:uid="{9EB5D030-E2AA-7F4B-A4DC-103EDFF22D70}" name="Provincia"/>
@@ -281,8 +278,8 @@
     <tableColumn id="15" xr3:uid="{05783EF8-12BB-8D46-966B-A6589486E222}" name="Parroquia"/>
     <tableColumn id="14" xr3:uid="{8011A1D5-CBA8-ED41-A8F1-D1686F2A01B5}" name="Dirección"/>
     <tableColumn id="7" xr3:uid="{B164287E-6857-0248-AF0F-65027DA44F51}" name="Zona de Movilidad"/>
-    <tableColumn id="8" xr3:uid="{1F32811C-5E6B-BC4D-AAC1-E5D291824B52}" name="Hogares a 5min"/>
-    <tableColumn id="9" xr3:uid="{1E3DC681-7CDD-C946-9434-58DF819DBB07}" name="Hogares a 10min"/>
+    <tableColumn id="8" xr3:uid="{1F32811C-5E6B-BC4D-AAC1-E5D291824B52}" name="Hogares 5min"/>
+    <tableColumn id="9" xr3:uid="{1E3DC681-7CDD-C946-9434-58DF819DBB07}" name="Hogares 10min"/>
     <tableColumn id="10" xr3:uid="{7586D6CF-1799-3542-B2B4-C15BB633A50A}" name="% NSE D"/>
     <tableColumn id="11" xr3:uid="{4337B1B0-EC8D-C148-A319-861109D19B25}" name="% NSE C-"/>
     <tableColumn id="12" xr3:uid="{383F9843-0D59-3245-92EE-EC16B6EABF1E}" name="% NSE C+"/>
@@ -293,14 +290,14 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{20D03861-84A2-1E4D-BB05-6E4FF6C62EB2}" name="Competencias" displayName="Competencias" ref="A1:G2" insertRow="1" totalsRowShown="0" headerRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{20D03861-84A2-1E4D-BB05-6E4FF6C62EB2}" name="Competencias" displayName="Competencias" ref="A1:G2" insertRow="1" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:G2" xr:uid="{20D03861-84A2-1E4D-BB05-6E4FF6C62EB2}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{FFBD8E60-590F-9746-8DCF-E4C3BC896D33}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{E47B1E6D-7385-9643-97B3-9B3B96443B43}" name="ID de Localidad"/>
+    <tableColumn id="2" xr3:uid="{E47B1E6D-7385-9643-97B3-9B3B96443B43}" name="Localidad ID"/>
     <tableColumn id="3" xr3:uid="{2D2B56D5-B326-B94D-A731-CC48092EC867}" name="Nombre"/>
-    <tableColumn id="4" xr3:uid="{86A5B628-E9B9-5A41-ABEB-8E0177B1912D}" name="Tipo de Competidor"/>
-    <tableColumn id="5" xr3:uid="{E4021B5A-E4D2-E746-B703-30CA2C6D9A84}" name="Tamaño (m²) "/>
+    <tableColumn id="4" xr3:uid="{86A5B628-E9B9-5A41-ABEB-8E0177B1912D}" name="Tipo"/>
+    <tableColumn id="5" xr3:uid="{E4021B5A-E4D2-E746-B703-30CA2C6D9A84}" name="Tamaño"/>
     <tableColumn id="6" xr3:uid="{3928116E-FEA8-C040-8B37-C514AA184C08}" name="Latitud"/>
     <tableColumn id="7" xr3:uid="{D34AE5FB-4C0C-9241-A362-4D6008160327}" name="Longitud"/>
   </tableColumns>
@@ -309,14 +306,14 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{5F83EA88-8AB2-664C-8F3D-377BDAF88C30}" name="Canibalizadores" displayName="Canibalizadores" ref="A1:G2" insertRow="1" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{5F83EA88-8AB2-664C-8F3D-377BDAF88C30}" name="Canibalizadores" displayName="Canibalizadores" ref="A1:G2" insertRow="1" totalsRowShown="0" headerRowDxfId="1">
   <autoFilter ref="A1:G2" xr:uid="{5F83EA88-8AB2-664C-8F3D-377BDAF88C30}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{710003A1-DD00-9448-B91D-C31FAC7440E1}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{A3AC0F3B-D3F2-6643-A8BD-03F69293ABE7}" name="ID de Localidad"/>
+    <tableColumn id="2" xr3:uid="{A3AC0F3B-D3F2-6643-A8BD-03F69293ABE7}" name="Localidad ID"/>
     <tableColumn id="3" xr3:uid="{F43FB2B6-5077-CD47-84BC-A2B7C9336BFF}" name="Nombre"/>
-    <tableColumn id="4" xr3:uid="{49826C52-3ECE-2A4A-A196-5F15ECAF6C2B}" name="Tipo de Competidor"/>
-    <tableColumn id="5" xr3:uid="{50D418F0-D71E-0244-829A-9B761C83F665}" name="Tamaño (m²) "/>
+    <tableColumn id="4" xr3:uid="{49826C52-3ECE-2A4A-A196-5F15ECAF6C2B}" name="Tipo"/>
+    <tableColumn id="5" xr3:uid="{50D418F0-D71E-0244-829A-9B761C83F665}" name="Tamaño"/>
     <tableColumn id="6" xr3:uid="{0DDD5804-35BA-BA4C-A0D2-30C71C05CDC2}" name="Latitud"/>
     <tableColumn id="7" xr3:uid="{53E5F83B-5EEF-0F44-8DAC-C042536C8872}" name="Longitud"/>
   </tableColumns>
@@ -684,49 +681,49 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="L1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" t="s">
-        <v>28</v>
-      </c>
-      <c r="J1" t="s">
-        <v>29</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="O1" t="s">
         <v>6</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>7</v>
       </c>
-      <c r="M1" t="s">
+      <c r="Q1" t="s">
         <v>8</v>
-      </c>
-      <c r="N1" t="s">
-        <v>9</v>
-      </c>
-      <c r="O1" t="s">
-        <v>10</v>
-      </c>
-      <c r="P1" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -776,22 +773,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -839,22 +836,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -899,49 +896,49 @@
   <sheetData>
     <row r="1" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>